<commit_message>
Correcting start year date part 2
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
+++ b/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\bldgs\BPSfDSPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150C21F9-C7F2-43C8-B4AC-6DBE0E8CB7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F40E33-0B4A-497B-A0A1-CD919E2C4959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="660" yWindow="240" windowWidth="19180" windowHeight="5820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32190" yWindow="4830" windowWidth="19200" windowHeight="11205" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="7" r:id="rId1"/>
@@ -501,109 +501,113 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AF7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.81640625" customWidth="1"/>
-    <col min="2" max="2" width="18.453125" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B1">
+        <v>2020</v>
+      </c>
+      <c r="C1">
         <v>2021</v>
       </c>
-      <c r="C1">
+      <c r="D1">
         <v>2022</v>
       </c>
-      <c r="D1">
+      <c r="E1">
         <v>2023</v>
       </c>
-      <c r="E1">
+      <c r="F1">
         <v>2024</v>
       </c>
-      <c r="F1">
+      <c r="G1">
         <v>2025</v>
       </c>
-      <c r="G1">
+      <c r="H1">
         <v>2026</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>2027</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>2028</v>
       </c>
-      <c r="J1">
+      <c r="K1">
         <v>2029</v>
       </c>
-      <c r="K1">
+      <c r="L1">
         <v>2030</v>
       </c>
-      <c r="L1">
+      <c r="M1">
         <v>2031</v>
       </c>
-      <c r="M1">
+      <c r="N1">
         <v>2032</v>
       </c>
-      <c r="N1">
+      <c r="O1">
         <v>2033</v>
       </c>
-      <c r="O1">
+      <c r="P1">
         <v>2034</v>
       </c>
-      <c r="P1">
+      <c r="Q1">
         <v>2035</v>
       </c>
-      <c r="Q1">
+      <c r="R1">
         <v>2036</v>
       </c>
-      <c r="R1">
+      <c r="S1">
         <v>2037</v>
       </c>
-      <c r="S1">
+      <c r="T1">
         <v>2038</v>
       </c>
-      <c r="T1">
+      <c r="U1">
         <v>2039</v>
       </c>
-      <c r="U1">
+      <c r="V1">
         <v>2040</v>
       </c>
-      <c r="V1">
+      <c r="W1">
         <v>2041</v>
       </c>
-      <c r="W1">
+      <c r="X1">
         <v>2042</v>
       </c>
-      <c r="X1">
+      <c r="Y1">
         <v>2043</v>
       </c>
-      <c r="Y1">
+      <c r="Z1">
         <v>2044</v>
       </c>
-      <c r="Z1">
+      <c r="AA1">
         <v>2045</v>
       </c>
-      <c r="AA1">
+      <c r="AB1">
         <v>2046</v>
       </c>
-      <c r="AB1">
+      <c r="AC1">
         <v>2047</v>
       </c>
-      <c r="AC1">
+      <c r="AD1">
         <v>2048</v>
       </c>
-      <c r="AD1">
+      <c r="AE1">
         <v>2049</v>
       </c>
-      <c r="AE1">
+      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -611,7 +615,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="5">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="D2" s="5">
         <v>0.15</v>
@@ -697,8 +701,11 @@
       <c r="AE2" s="5">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="AF2" s="5">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -706,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="5">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="D3" s="5">
         <v>0.15</v>
@@ -792,8 +799,11 @@
       <c r="AE3" s="5">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="AF3" s="5">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -801,7 +811,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="5">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="D4" s="5">
         <v>0.15</v>
@@ -887,15 +897,19 @@
       <c r="AE4" s="5">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="AF4" s="5">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="B5" s="3"/>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="B7" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="C7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -904,6 +918,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002041A8AB53924247A2770D65450F5227" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="90fff4f083191fe75a03dbd50c7739fc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1659011e-6b88-4225-9a61-aaf33aaf19e8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7fee88694a371868130ae0617c69143c" ns2:_="">
     <xsd:import namespace="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
@@ -1047,12 +1067,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1063,6 +1077,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F020338D-1674-4302-A6BE-E8EA0F4ACDBC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CD04559-E101-41C1-865F-CB5F5B537630}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1080,15 +1103,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F020338D-1674-4302-A6BE-E8EA0F4ACDBC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BC8B6BD-8498-457E-9CD1-92EA964F629C}">
   <ds:schemaRefs>

</xml_diff>